<commit_message>
Working Crossref metadata extraction for all journals using CloudScraper
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -836,754 +836,1165 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Translational Psychiatry</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>10.1038/s41398-025-03398-0</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>['Francesca McEwan', 'Chiho Kambara', 'Jarred M. Lorusso', 'Michael K. Harte', 'Jocelyn D. Glazier', 'Reinmar Hager']</t>
-        </is>
-      </c>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>['Omar Soler-Cedeno', 'Ewa Galaj', 'Benjamin Klein', 'Jianjing Cao', 'Guo-Hua Bi', 'Amy Hauck Newman', 'Zheng-Xiong Xi']</t>
+          <t>['Gaoyu Liu', 'Huachen Huang', 'Ying Wang', 'Yali Han', 'Jianye Wang', 'Mengxuan Shi', 'Pan Zhou', 'Chun Chen', 'Ying Yu', 'Qiang Liu', 'Jie Zhou']</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
+          <t>Activity-dependent development of the body’s touch receptors</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03401-8</t>
+          <t>10.1016/j.neuron.2025.04.015</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>['Andreas Walther', 'Lukas Eggenberger', 'Rudolf Debelak', 'Clemens Kirschbaum', 'Isabelle Häberling', 'Ester Osuna', 'Michael Strumberger', 'Susanne Walitza', 'Jeannine Baumgartner', 'Isabelle Herter-Aeberli', 'Gregor Berger']</t>
+          <t>['Celine Santiago', 'Julianna Siegrist', 'Nusrat Africawala', 'Annie Handler', 'Aniqa Tasnim', 'Rabia Anjum', 'Josef Turecek', 'Brendan P. Lehnert', 'Sophia Renauld', 'Jinheon Choi', 'Michael Nolan-Tamariz', 'Michael Iskols', 'Alexandra R. Magee', 'Suzanne Paradis', 'Nikhil Sharma', 'David D. Ginty']</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03390-8</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>['Claire A. Lavalley', 'Marishka M. Mehta', 'Samuel Taylor', 'Anne E. Chuning', 'Jennifer L. Stewart', 'Quentin J. M. Huys', 'Sahib S. Khalsa', 'Martin P. Paulus', 'Ryan Smith']</t>
+          <t>['Wenrui Xie', 'Debora Denardin Lückemeyer', 'Katherine A. Qualls', 'Arthur Silveira Prudente', 'Temugin Berta', 'Mingxia Gu', 'Judith A. Strong', 'Xinzhong Dong', 'Jun-Ming Zhang']</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03393-5</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>['Yi-An Hung', 'Tien-Chueh Kuo', 'Yufeng Jane Tseng', 'Chi-Yung Shang', 'Susan Shur-Fen Gau']</t>
+          <t>['Tianming Li', 'Wenjie Zhou', 'Jin Ke', 'Matthew Chen', 'Zhen Wang', 'Lauren Hayashi', 'Xiaojing Su', 'Wenbin Jia', 'Wenxi Huang', 'Chien-Sheng Wang', 'Kapsa Bengyella', 'Yang Yang', 'Rafael Hernandez', 'Yan Zhang', 'Xinglei Song', 'Tianle Xu', 'Tianwen Huang', 'Yuanyuan Liu']</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03393-5</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>['Yi-An Hung', 'Tien-Chueh Kuo', 'Yufeng Jane Tseng', 'Chi-Yung Shang', 'Susan Shur-Fen Gau']</t>
+          <t>['Adam P. Caccavano', 'Anna Vlachos', 'Nadiya McLean', 'Sarah Kimmel', 'June Hoan Kim', 'Geoffrey Vargish', 'Vivek Mahadevan', 'Lauren Hewitt', 'Anthony M. Rossi', 'Ilona Spineux', 'Sherry Jingjing Wu', 'Elisabetta Furlanis', 'Min Dai', 'Brenda Leyva Garcia', 'Yating Wang', 'Ramesh Chittajallu', 'Edra London', 'Xiaoqing Yuan', 'Steven Hunt', 'Daniel Abebe', 'Mark A.G. Eldridge', 'Alex C. Cummins', 'Brendan E. Hines', 'Anya Plotnikova', 'Arya Mohanty', 'Bruno B. Averbeck', 'Kareem A. Zaghloul', 'Jordane Dimidschstein', 'Gord Fishell', 'Kenneth A. Pelkey', 'Chris J. McBain']</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
+          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03322-6</t>
+          <t>10.1016/j.neuron.2025.03.018</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>['Yanzhi Li', 'Liwan Zhu', 'Yang Yang', 'Caiyun Zhang', 'Hao Zhao', 'Jingman Shi', 'Wenjian Lai', 'Wenjing Zhou', 'Guangduoji Shi', 'Wanxin Wang', 'Lan Guo', 'Ciyong Lu']</t>
+          <t>['Qingtao Sun', 'Mingzhe Liu', 'Wuqiang Guan', 'Xiong Xiao', 'Chunyang Dong', 'Michael R. Bruchas', 'Larry S. Zweifel', 'Yulong Li', 'Lin Tian', 'Bo Li']</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03399-z</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>['Veronica Rivi', 'Pierfrancesco Sarti', 'Istvan Fodor', 'Zsolt Pirger', 'Joris M. Koene', 'Luca Pani', 'Anuradha Batabyal', 'Ken Lukowiak', 'Johanna Maria Catharina Blom', 'Fabio Tascedda', 'Cristina Benatti']</t>
+          <t>['Lindsay A. Hohsfield', 'Sung Jin Kim', 'Rocio A. Barahona', 'Caden M. Henningfield', 'Kimiya Mansour', 'Kristen D. Vallejo', 'Kate I. Tsourmas', 'Nellie E. Kwang', 'Yasamine Ghorbanian', 'Julio Alejandro Ayala Angulo', 'Pan Gao', 'Collin Pachow', 'Matthew A. Inlay', 'Craig M. Walsh', 'Xiangmin Xu', 'Thomas E. Lane', 'Kim N. Green']</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
+          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03392-6</t>
+          <t>10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>['Christelle Langley', 'Graham K. Murray', 'Sophia Armand', 'Franziska Knolle', 'Rudolf N. Cardinal', 'Annette Johansen', 'Peter S. Jensen', 'Jianfeng Feng', 'Dea S. Stenbæk', 'Gitte M. Knudsen', 'Patrick M. Fisher', 'Barbara J. Sahakian']</t>
+          <t>['Charles Ducrot', 'Adèle Drouet', 'Béatrice Tessier', 'Chloé Desquines', 'Tiffany Cloâtre', 'Rania-Cérine Mazouzi', 'Florian Levet', 'Alexandre Favereaux', 'Mathieu Letellier', 'Olivier Thoumine']</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
+          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03272-z</t>
+          <t>10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>['Maryse J. Luijendijk', 'Margot E. T. Tesselaar', 'Huub H. van Rossum', 'Martijn van Faassen', 'Catharina M. Korse', 'Wieke H. M. Verbeek', 'Jocelyn R. Spruit', 'Pernilla C. Scheelings', 'Eva H. Hooghiemstra', 'Ido P. Kema', 'Henricus G. Ruhé', 'Sanne B. Schagen', 'Froukje E. de Vries']</t>
+          <t>['Megan M. Davis', 'Mackenzie Woodburn', 'Tehila Nugiel', 'Divyangana Rakesh', 'Maresa Tate', 'William Asciutto', 'Weili Lin', 'Jessica R. Cohen', 'Margaret A. Sheridan']</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>['Aljoscha Nern', 'Frank Loesche', 'Shin-ya Takemura', 'Laura E. Burnett', 'Marisa Dreher', 'Eyal Gruntman', 'Judith Hoeller', 'Gary B. Huang', 'Michał Januszewski', 'Nathan C. Klapoetke', 'Sanna Koskela', 'Kit D. Longden', 'Zhiyuan Lu', 'Stephan Preibisch', 'Wei Qiu', 'Edward M. Rogers', 'Pavithraa Seenivasan', 'Arthur Zhao', 'John Bogovic', 'Brandon S. Canino', 'Jody Clements', 'Michael Cook', 'Samantha Finley-May', 'Miriam A. Flynn', 'Imran Hameed', 'Alexandra M. C. Fragniere', 'Kenneth J. Hayworth', 'Gary Patrick Hopkins', 'Philip M. Hubbard', 'William T. Katz', 'Julie Kovalyak', 'Shirley A. Lauchie', 'Meghan Leonard', 'Alanna Lohff', 'Charli A. Maldonado', 'Caroline Mooney', 'Nneoma Okeoma', 'Donald J. Olbris', 'Christopher Ordish', 'Tyler Paterson', 'Emily M. Phillips', 'Tobias Pietzsch', 'Jennifer Rivas Salinas', 'Patricia K. Rivlin', 'Philipp Schlegel', 'Ashley L. Scott', 'Louis A. Scuderi', 'Satoko Takemura', 'Iris Talebi', 'Alexander Thomson', 'Eric T. Trautman', 'Lowell Umayam', 'Claire Walsh', 'John J. Walsh', 'C. Shan Xu', 'Emily A. Yakal', 'Tansy Yang', 'Ting Zhao', 'Jan Funke', 'Reed George', 'Harald F. Hess', 'Gregory S. X. E. Jefferis', 'Christopher Knecht', 'Wyatt Korff', 'Stephen M. Plaza', 'Sandro Romani', 'Stephan Saalfeld', 'Louis K. Scheffer', 'Stuart Berg', 'Gerald M. Rubin', 'Michael B. Reiser']</t>
+          <t>['Karthik Srinivasan', 'Eric Lowet', 'Bruno Gomes', 'Robert Desimone']</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Psychedelic control of neuroimmune interactions governing fear</t>
+          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08880-9</t>
+          <t>10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>['Elizabeth N. Chung', 'Jinsu Lee', 'Carolina M. Polonio', 'Joshua Choi', 'Camilo Faust Akl', 'Michael Kilian', 'Wiebke M. Weiß', 'Georgia Gunner', 'Mingyu Ye', 'Tae Hyun Heo', 'Sienna S. Drake', 'Liu Yang', 'Catarina R. G. L. d’Eca', 'Joon-Hyuk Lee', 'Liwen Deng', 'Daniel Farrenkopf', 'Anton M. Schüle', 'Hong-Gyun Lee', 'Oreoluwa Afolabi', 'Sharmin Ghaznavi', 'Stelios M. Smirnakis', 'Isaac M. Chiu', 'Vijay K. Kuchroo', 'Francisco J. Quintana', 'Michael A. Wheeler']</t>
+          <t>['Wei Wen', 'Adriana M. Prada', 'Gina G. Turrigiano']</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
+          <t>Grouping signals in primate visual cortex</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.003</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>['Rikard Frederiksen', 'Paul J. Bonezzi', 'Gordon L. Fain', 'Alapakkam P. Sampath']</t>
+          <t>['Tom P. Franken', 'John H. Reynolds']</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
+          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1139-24.2025</t>
+          <t>10.1038/s41398-025-03398-0</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>['Paula T. Kuokkanen', 'Ira Kraemer', 'Christine Köppl', 'Catherine E. Carr', 'Richard Kempter']</t>
+          <t>['Francesca McEwan', 'Chiho Kambara', 'Jarred M. Lorusso', 'Michael K. Harte', 'Jocelyn D. Glazier', 'Reinmar Hager']</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0217-25.2025</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>['Paola Alemán-Andrade', 'Menno P. Witter', 'Ken-Ichiro Tsutsui', 'Shinya Ohara']</t>
+          <t>['Omar Soler-Cedeno', 'Ewa Galaj', 'Benjamin Klein', 'Jianjing Cao', 'Guo-Hua Bi', 'Amy Hauck Newman', 'Zheng-Xiong Xi']</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
+          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2325-24.2025</t>
+          <t>10.1038/s41398-025-03401-8</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>['James B. Whitley', 'Sean P. Masterson', 'Thomas Gordon', 'Kyle L. Whyland', 'Peter W. Campbell', 'Na Zhou', 'Gubbi Govindaiah', 'William Guido', 'Martha E. Bickford']</t>
+          <t>['Andreas Walther', 'Lukas Eggenberger', 'Rudolf Debelak', 'Clemens Kirschbaum', 'Isabelle Häberling', 'Ester Osuna', 'Michael Strumberger', 'Susanne Walitza', 'Jeannine Baumgartner', 'Isabelle Herter-Aeberli', 'Gregor Berger']</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
+          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1001-24.2025</t>
+          <t>10.1038/s41398-025-03390-8</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>['Carolina Fernandes-Henriques', 'Yuval Guetta', 'Mia G. Sclar', 'Rebecca Zhang', 'Yuka Miura', 'Katherine R. Surrence', 'Allyson K. Friedman', 'Ekaterina Likhtik']</t>
+          <t>['Claire A. Lavalley', 'Marishka M. Mehta', 'Samuel Taylor', 'Anne E. Chuning', 'Jennifer L. Stewart', 'Quentin J. M. Huys', 'Sahib S. Khalsa', 'Martin P. Paulus', 'Ryan Smith']</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
+          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1876-24.2025</t>
+          <t>10.1038/s41398-025-03393-5</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>['Lidon Marin-Marin', 'Susanne Eisenhauer', 'Tirso R. J. Gonzalez Alam', 'Daniel S. Margulies', 'Jonathan Smallwood', 'Elizabeth Jefferies']</t>
+          <t>['Yi-An Hung', 'Tien-Chueh Kuo', 'Yufeng Jane Tseng', 'Chi-Yung Shang', 'Susan Shur-Fen Gau']</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
+          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2187-24.2025</t>
+          <t>10.1038/s41398-025-03393-5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>['Min Wu', 'Marleen J. Schoenfeld', 'Carl Lindersson', 'Sven Braeutigam', 'Catharina Zich', 'Charlotte J. Stagg']</t>
+          <t>['Yi-An Hung', 'Tien-Chueh Kuo', 'Yufeng Jane Tseng', 'Chi-Yung Shang', 'Susan Shur-Fen Gau']</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1038/s41398-025-03322-6</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>['Marie-Lucie Read', 'Carl J. Hodgetts', 'Andrew D. Lawrence', 'C. John Evans', 'Krish D. Singh', 'Katja Umla-Runge', 'Kim S. Graham']</t>
+          <t>['Yanzhi Li', 'Liwan Zhu', 'Yang Yang', 'Caiyun Zhang', 'Hao Zhao', 'Jingman Shi', 'Wenjian Lai', 'Wenjing Zhou', 'Guangduoji Shi', 'Wanxin Wang', 'Lan Guo', 'Ciyong Lu']</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
+          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2378-24.2025</t>
+          <t>10.1038/s41398-025-03399-z</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>['Marie Levorsen', 'Ryuta Aoki', 'Constantine Sedikides', 'Keise Izuma']</t>
+          <t>['Veronica Rivi', 'Pierfrancesco Sarti', 'Istvan Fodor', 'Zsolt Pirger', 'Joris M. Koene', 'Luca Pani', 'Anuradha Batabyal', 'Ken Lukowiak', 'Johanna Maria Catharina Blom', 'Fabio Tascedda', 'Cristina Benatti']</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
+          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
+          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0044-25.2025</t>
+          <t>10.1038/s41398-025-03392-6</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>['Puti Wen', 'Lowell W. Thompson', 'Ari Rosenberg', 'Michael S. Landy', 'Bas Rokers']</t>
+          <t>['Christelle Langley', 'Graham K. Murray', 'Sophia Armand', 'Franziska Knolle', 'Rudolf N. Cardinal', 'Annette Johansen', 'Peter S. Jensen', 'Jianfeng Feng', 'Dea S. Stenbæk', 'Gitte M. Knudsen', 'Patrick M. Fisher', 'Barbara J. Sahakian']</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
+          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2186-24.2025</t>
+          <t>10.1038/s41398-025-03272-z</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>['Siyi Chen (陈思佚)', 'Nika Merkuš', 'Shao-Yang Tsai (蔡劭扬)', 'Si Cheng (程思)', 'Hermann J. Müller', 'Zhuanghua Shi (施壮华)']</t>
+          <t>['Maryse J. Luijendijk', 'Margot E. T. Tesselaar', 'Huub H. van Rossum', 'Martijn van Faassen', 'Catharina M. Korse', 'Wieke H. M. Verbeek', 'Jocelyn R. Spruit', 'Pernilla C. Scheelings', 'Eva H. Hooghiemstra', 'Ido P. Kema', 'Henricus G. Ruhé', 'Sanne B. Schagen', 'Froukje E. de Vries']</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>The Journal of Neuroscience</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>['Reut Hazani', 'Jocelyn M. Breton', 'Estherina Trachtenberg', 'Keren Ruzal', 'Bar Shvalbo', 'Ben Kantor', 'Adva Maman', 'Einat Bigelman', 'Steve Cole', 'Aron Weller', 'Inbal Ben-Ami Bartal']</t>
-        </is>
-      </c>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>['Yan Chen', 'Xiangyue Xiao', 'Zhicai Dong', 'Junhua Ding', 'Sara Cruz', 'Ming Zhang', 'Yuhan Lu', 'Nai Ding', 'Charlène Aubinet', 'Steven Laureys', 'Haibo Di']</t>
+          <t>['Aljoscha Nern', 'Frank Loesche', 'Shin-ya Takemura', 'Laura E. Burnett', 'Marisa Dreher', 'Eyal Gruntman', 'Judith Hoeller', 'Gary B. Huang', 'Michał Januszewski', 'Nathan C. Klapoetke', 'Sanna Koskela', 'Kit D. Longden', 'Zhiyuan Lu', 'Stephan Preibisch', 'Wei Qiu', 'Edward M. Rogers', 'Pavithraa Seenivasan', 'Arthur Zhao', 'John Bogovic', 'Brandon S. Canino', 'Jody Clements', 'Michael Cook', 'Samantha Finley-May', 'Miriam A. Flynn', 'Imran Hameed', 'Alexandra M. C. Fragniere', 'Kenneth J. Hayworth', 'Gary Patrick Hopkins', 'Philip M. Hubbard', 'William T. Katz', 'Julie Kovalyak', 'Shirley A. Lauchie', 'Meghan Leonard', 'Alanna Lohff', 'Charli A. Maldonado', 'Caroline Mooney', 'Nneoma Okeoma', 'Donald J. Olbris', 'Christopher Ordish', 'Tyler Paterson', 'Emily M. Phillips', 'Tobias Pietzsch', 'Jennifer Rivas Salinas', 'Patricia K. Rivlin', 'Philipp Schlegel', 'Ashley L. Scott', 'Louis A. Scuderi', 'Satoko Takemura', 'Iris Talebi', 'Alexander Thomson', 'Eric T. Trautman', 'Lowell Umayam', 'Claire Walsh', 'John J. Walsh', 'C. Shan Xu', 'Emily A. Yakal', 'Tansy Yang', 'Ting Zhao', 'Jan Funke', 'Reed George', 'Harald F. Hess', 'Gregory S. X. E. Jefferis', 'Christopher Knecht', 'Wyatt Korff', 'Stephen M. Plaza', 'Sandro Romani', 'Stephan Saalfeld', 'Louis K. Scheffer', 'Stuart Berg', 'Gerald M. Rubin', 'Michael B. Reiser']</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Psychedelic control of neuroimmune interactions governing fear</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1038/s41586-025-08880-9</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>['Sai Yasukochi', 'Wakaba Yamakawa', 'Marie Taniguchi', 'Sayaka Itoyama', 'Akito Tsuruta', 'Naoki Kusunose', 'Tomoaki Yamauchi', 'Risako Nakamura', 'Naoya Matsunaga', 'Shigehiro Ohdo', 'Satoru Koyanagi']</t>
+          <t>['Elizabeth N. Chung', 'Jinsu Lee', 'Carolina M. Polonio', 'Joshua Choi', 'Camilo Faust Akl', 'Michael Kilian', 'Wiebke M. Weiß', 'Georgia Gunner', 'Mingyu Ye', 'Tae Hyun Heo', 'Sienna S. Drake', 'Liu Yang', 'Catarina R. G. L. d’Eca', 'Joon-Hyuk Lee', 'Liwen Deng', 'Daniel Farrenkopf', 'Anton M. Schüle', 'Hong-Gyun Lee', 'Oreoluwa Afolabi', 'Sharmin Ghaznavi', 'Stelios M. Smirnakis', 'Isaac M. Chiu', 'Vijay K. Kuchroo', 'Francisco J. Quintana', 'Michael A. Wheeler']</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>A neural basis for distinguishing imagination from reality</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1016/j.neuron.2025.05.015</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>['Xiaodong Xu', 'Cheng Jia', 'Kang Chen', 'Lijuan Chen']</t>
+          <t>['Nadine Dijkstra', 'Thomas von Rein', 'Peter Kok', 'Stephen M. Fleming']</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Neuron</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>10.1016/j.neuron.2025.05.009</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>['Wang Zheng', 'Augustus J. Lowry', 'Harper E. Smith', 'Jiale Xie', 'Shaun Rawson', 'Chen Wang', 'Jin Ou', 'Marcos Sotomayor', 'Tian-Min Fu', 'Huanghe Yang', 'Jeffrey R. Holt']</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.1920-24.2025</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>['Rikard Frederiksen', 'Paul J. Bonezzi', 'Gordon L. Fain', 'Alapakkam P. Sampath']</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.1139-24.2025</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>['Paula T. Kuokkanen', 'Ira Kraemer', 'Christine Köppl', 'Catherine E. Carr', 'Richard Kempter']</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.0217-25.2025</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>['Paola Alemán-Andrade', 'Menno P. Witter', 'Ken-Ichiro Tsutsui', 'Shinya Ohara']</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.2325-24.2025</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>['James B. Whitley', 'Sean P. Masterson', 'Thomas Gordon', 'Kyle L. Whyland', 'Peter W. Campbell', 'Na Zhou', 'Gubbi Govindaiah', 'William Guido', 'Martha E. Bickford']</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.1001-24.2025</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>['Carolina Fernandes-Henriques', 'Yuval Guetta', 'Mia G. Sclar', 'Rebecca Zhang', 'Yuka Miura', 'Katherine R. Surrence', 'Allyson K. Friedman', 'Ekaterina Likhtik']</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.1876-24.2025</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>['Lidon Marin-Marin', 'Susanne Eisenhauer', 'Tirso R. J. Gonzalez Alam', 'Daniel S. Margulies', 'Jonathan Smallwood', 'Elizabeth Jefferies']</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.2187-24.2025</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>['Min Wu', 'Marleen J. Schoenfeld', 'Carl Lindersson', 'Sven Braeutigam', 'Catharina Zich', 'Charlotte J. Stagg']</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>['Marie-Lucie Read', 'Carl J. Hodgetts', 'Andrew D. Lawrence', 'C. John Evans', 'Krish D. Singh', 'Katja Umla-Runge', 'Kim S. Graham']</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.2378-24.2025</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>['Marie Levorsen', 'Ryuta Aoki', 'Constantine Sedikides', 'Keise Izuma']</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.0044-25.2025</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>['Puti Wen', 'Lowell W. Thompson', 'Ari Rosenberg', 'Michael S. Landy', 'Bas Rokers']</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.2186-24.2025</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>['Siyi Chen (陈思佚)', 'Nika Merkuš', 'Shao-Yang Tsai (蔡劭扬)', 'Si Cheng (程思)', 'Hermann J. Müller', 'Zhuanghua Shi (施壮华)']</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>['Reut Hazani', 'Jocelyn M. Breton', 'Estherina Trachtenberg', 'Keren Ruzal', 'Bar Shvalbo', 'Ben Kantor', 'Adva Maman', 'Einat Bigelman', 'Steve Cole', 'Aron Weller', 'Inbal Ben-Ami Bartal']</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>['Yan Chen', 'Xiangyue Xiao', 'Zhicai Dong', 'Junhua Ding', 'Sara Cruz', 'Ming Zhang', 'Yuhan Lu', 'Nai Ding', 'Charlène Aubinet', 'Steven Laureys', 'Haibo Di']</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>['Sai Yasukochi', 'Wakaba Yamakawa', 'Marie Taniguchi', 'Sayaka Itoyama', 'Akito Tsuruta', 'Naoki Kusunose', 'Tomoaki Yamauchi', 'Risako Nakamura', 'Naoya Matsunaga', 'Shigehiro Ohdo', 'Satoru Koyanagi']</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>npj Science of Learning</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>10.1038/s41539-025-00327-0</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>['Xiaodong Xu', 'Cheng Jia', 'Kang Chen', 'Lijuan Chen']</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>npj Science of Learning</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>['Christoph Bamberg', 'Sarah Weigelt', 'Klara Hagelweide']</t>
         </is>

</xml_diff>

<commit_message>
Added protection against IP blocking (rotating headers, randomised wait times). Improved DOI extraction/Crossref metadata to work for all journals (previously did not work for Science). Email extraction pending.
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1464242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -468,24 +468,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Synergistic Reinforcement Learning by Cooperation of the Cerebellum and Basal Ganglia</t>
+          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1464-24.2025</t>
+          <t>10.1523/JNEUROSCI.0436-25.2025</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>['Tatsumi Yoshida', 'Hikaru Sugino', 'Hinako Yamamoto', 'Sho Tanno', 'Mikihide Tamura', 'Jun Igarashi', 'Yoshikazu Isomura', 'Riichiro Hira']</t>
+          <t>['Jingyi Yang', 'Krystel Huxlin', 'Farran Briggs']</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -495,24 +495,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
+          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0436-25.2025</t>
+          <t>10.1523/JNEUROSCI.1907-24.2025</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>['Jingyi Yang', 'Krystel Huxlin', 'Farran Briggs']</t>
+          <t>['Johanna B. Fritzinger', 'Laurel H. Carney']</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -522,24 +522,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
+          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1907-24.2025</t>
+          <t>10.1523/JNEUROSCI.2218-24.2025</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>['Johanna B. Fritzinger', 'Laurel H. Carney']</t>
+          <t>['Huan Gao', 'Sandhya Ramachandran', 'Kai Yu', 'Bin He']</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -549,24 +549,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
+          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2218-24.2025</t>
+          <t>10.1523/JNEUROSCI.0491-25.2025</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>['Huan Gao', 'Sandhya Ramachandran', 'Kai Yu', 'Bin He']</t>
+          <t>['Wenliang Wang', 'Mark A. G. Eldridge', 'Tsuyoshi Setogawa', 'Spencer Webster-Bass', 'Nanami Miyazaki', 'Jonah E. Pearl', 'Jeih-San Liow', 'Walter Lerchner', 'Bing Li', 'Janita N. Turchi', 'Sanjay Telu', 'Sridhar Goud Nerella', 'Phelix Rodriguez', 'Robert B. Innis', 'Victor W. Pike', 'Bruno B. Averbeck', 'Barry J. Richmond']</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -576,24 +576,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0491-25.2025</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>['Wenliang Wang', 'Mark A. G. Eldridge', 'Tsuyoshi Setogawa', 'Spencer Webster-Bass', 'Nanami Miyazaki', 'Jonah E. Pearl', 'Jeih-San Liow', 'Walter Lerchner', 'Bing Li', 'Janita N. Turchi', 'Sanjay Telu', 'Sridhar Goud Nerella', 'Phelix Rodriguez', 'Robert B. Innis', 'Victor W. Pike', 'Bruno B. Averbeck', 'Barry J. Richmond']</t>
+          <t>['Jae-Chang Kim', 'Lydia Hellrung', 'Stephan Nebe', 'Philippe N. Tobler']</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -603,24 +603,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>['Jae-Chang Kim', 'Lydia Hellrung', 'Stephan Nebe', 'Philippe N. Tobler']</t>
+          <t>['Tilman Stephani', 'Arno Villringer', 'Vadim V. Nikulin']</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -630,24 +630,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1523/JNEUROSCI.1788-24.2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>['Tilman Stephani', 'Arno Villringer', 'Vadim V. Nikulin']</t>
+          <t>['Lihan Cui', 'Ke Bo', 'Changhao Xiong', 'Yujun Chen', 'Andreas Keil', 'Mingzhou Ding']</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -657,24 +657,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
+          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1788-24.2025</t>
+          <t>10.1523/JNEUROSCI.0404-25.2025</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>['Lihan Cui', 'Ke Bo', 'Changhao Xiong', 'Yujun Chen', 'Andreas Keil', 'Mingzhou Ding']</t>
+          <t>['Elana R. Goldenkoff', 'James A. Brissenden', 'Taraz G. Lee', 'Katherine J. Michon', 'Michael Vesia']</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -684,24 +684,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
+          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0404-25.2025</t>
+          <t>10.1523/JNEUROSCI.1114-24.2025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>['Elana R. Goldenkoff', 'James A. Brissenden', 'Taraz G. Lee', 'Katherine J. Michon', 'Michael Vesia']</t>
+          <t>['JuYoung Kim', 'Hackjin Kim']</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -711,24 +711,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
+          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1114-24.2025</t>
+          <t>10.1523/JNEUROSCI.1920-23.2025</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>['JuYoung Kim', 'Hackjin Kim']</t>
+          <t>['Dilara Berkay', 'Adrianna C. Jenkins']</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -738,24 +738,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-23.2025</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>['Dilara Berkay', 'Adrianna C. Jenkins']</t>
+          <t>['Adam Steel', 'Deepasri Prasad', 'Brenda D. Garcia', 'Caroline E. Robertson']</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -765,24 +765,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>['Adam Steel', 'Deepasri Prasad', 'Brenda D. Garcia', 'Caroline E. Robertson']</t>
+          <t>['Ziqi Liang', 'Junjie Wu', 'Qiang Liu', 'Dezhe Qin', 'Min Wang', 'Xiaofen Zhong', 'Weixiang Guo']</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -792,62 +792,78 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>['Ziqi Liang', 'Junjie Wu', 'Qiang Liu', 'Dezhe Qin', 'Min Wang', 'Xiaofen Zhong', 'Weixiang Guo']</t>
+          <t>['Takahiro Morito', 'Shoko Hashimoto', 'Risa Takamura', 'Naoto Watamura', 'Naomasa Kakiya', 'Ryo Fujioka', 'Naomi Mihara', 'Misaki Sekiguchi', 'Kaori Watanabe-Iwata', 'Naoko Kamano', 'Mohan Qi', 'Yukio Matsuba', 'Satoshi Tsubuki', 'Takashi Saito', 'Nobuhisa Iwata', 'Hiroki Sasaguri', 'Takaomi C. Saido']</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>['Takahiro Morito', 'Shoko Hashimoto', 'Risa Takamura', 'Naoto Watamura', 'Naomasa Kakiya', 'Ryo Fujioka', 'Naomi Mihara', 'Misaki Sekiguchi', 'Kaori Watanabe-Iwata', 'Naoko Kamano', 'Mohan Qi', 'Yukio Matsuba', 'Satoshi Tsubuki', 'Takashi Saito', 'Nobuhisa Iwata', 'Hiroki Sasaguri', 'Takaomi C. Saido']</t>
+          <t>['Yuliang Han', 'Juan Li', 'Wencheng Xia', 'Qintong Li', 'Zihan Sun', 'Wen Zeng', 'Yingxin Hu', 'Kelvin C. Luk', 'Cong Liu', 'ShengQi Xiang', 'Zhuohao He']</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Neuron</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>10.1016/j.neuron.2025.03.014</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>['Gaoyu Liu', 'Huachen Huang', 'Ying Wang', 'Yali Han', 'Jianye Wang', 'Mengxuan Shi', 'Pan Zhou', 'Chun Chen', 'Ying Yu', 'Qiang Liu', 'Jie Zhou']</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -857,24 +873,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Activity-dependent development of the body’s touch receptors</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1016/j.neuron.2025.04.015</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>['Gaoyu Liu', 'Huachen Huang', 'Ying Wang', 'Yali Han', 'Jianye Wang', 'Mengxuan Shi', 'Pan Zhou', 'Chun Chen', 'Ying Yu', 'Qiang Liu', 'Jie Zhou']</t>
+          <t>['Celine Santiago', 'Julianna Siegrist', 'Nusrat Africawala', 'Annie Handler', 'Aniqa Tasnim', 'Rabia Anjum', 'Josef Turecek', 'Brendan P. Lehnert', 'Sophia Renauld', 'Jinheon Choi', 'Michael Nolan-Tamariz', 'Michael Iskols', 'Alexandra R. Magee', 'Suzanne Paradis', 'Nikhil Sharma', 'David D. Ginty']</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -884,24 +900,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Activity-dependent development of the body’s touch receptors</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.04.015</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>['Celine Santiago', 'Julianna Siegrist', 'Nusrat Africawala', 'Annie Handler', 'Aniqa Tasnim', 'Rabia Anjum', 'Josef Turecek', 'Brendan P. Lehnert', 'Sophia Renauld', 'Jinheon Choi', 'Michael Nolan-Tamariz', 'Michael Iskols', 'Alexandra R. Magee', 'Suzanne Paradis', 'Nikhil Sharma', 'David D. Ginty']</t>
+          <t>['Wenrui Xie', 'Debora Denardin Lückemeyer', 'Katherine A. Qualls', 'Arthur Silveira Prudente', 'Temugin Berta', 'Mingxia Gu', 'Judith A. Strong', 'Xinzhong Dong', 'Jun-Ming Zhang']</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -911,24 +927,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>['Wenrui Xie', 'Debora Denardin Lückemeyer', 'Katherine A. Qualls', 'Arthur Silveira Prudente', 'Temugin Berta', 'Mingxia Gu', 'Judith A. Strong', 'Xinzhong Dong', 'Jun-Ming Zhang']</t>
+          <t>['Tianming Li', 'Wenjie Zhou', 'Jin Ke', 'Matthew Chen', 'Zhen Wang', 'Lauren Hayashi', 'Xiaojing Su', 'Wenbin Jia', 'Wenxi Huang', 'Chien-Sheng Wang', 'Kapsa Bengyella', 'Yang Yang', 'Rafael Hernandez', 'Yan Zhang', 'Xinglei Song', 'Tianle Xu', 'Tianwen Huang', 'Yuanyuan Liu']</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -938,24 +954,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>['Tianming Li', 'Wenjie Zhou', 'Jin Ke', 'Matthew Chen', 'Zhen Wang', 'Lauren Hayashi', 'Xiaojing Su', 'Wenbin Jia', 'Wenxi Huang', 'Chien-Sheng Wang', 'Kapsa Bengyella', 'Yang Yang', 'Rafael Hernandez', 'Yan Zhang', 'Xinglei Song', 'Tianle Xu', 'Tianwen Huang', 'Yuanyuan Liu']</t>
+          <t>['Adam P. Caccavano', 'Anna Vlachos', 'Nadiya McLean', 'Sarah Kimmel', 'June Hoan Kim', 'Geoffrey Vargish', 'Vivek Mahadevan', 'Lauren Hewitt', 'Anthony M. Rossi', 'Ilona Spineux', 'Sherry Jingjing Wu', 'Elisabetta Furlanis', 'Min Dai', 'Brenda Leyva Garcia', 'Yating Wang', 'Ramesh Chittajallu', 'Edra London', 'Xiaoqing Yuan', 'Steven Hunt', 'Daniel Abebe', 'Mark A.G. Eldridge', 'Alex C. Cummins', 'Brendan E. Hines', 'Anya Plotnikova', 'Arya Mohanty', 'Bruno B. Averbeck', 'Kareem A. Zaghloul', 'Jordane Dimidschstein', 'Gord Fishell', 'Kenneth A. Pelkey', 'Chris J. McBain']</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -965,24 +981,24 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1016/j.neuron.2025.03.018</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>['Adam P. Caccavano', 'Anna Vlachos', 'Nadiya McLean', 'Sarah Kimmel', 'June Hoan Kim', 'Geoffrey Vargish', 'Vivek Mahadevan', 'Lauren Hewitt', 'Anthony M. Rossi', 'Ilona Spineux', 'Sherry Jingjing Wu', 'Elisabetta Furlanis', 'Min Dai', 'Brenda Leyva Garcia', 'Yating Wang', 'Ramesh Chittajallu', 'Edra London', 'Xiaoqing Yuan', 'Steven Hunt', 'Daniel Abebe', 'Mark A.G. Eldridge', 'Alex C. Cummins', 'Brendan E. Hines', 'Anya Plotnikova', 'Arya Mohanty', 'Bruno B. Averbeck', 'Kareem A. Zaghloul', 'Jordane Dimidschstein', 'Gord Fishell', 'Kenneth A. Pelkey', 'Chris J. McBain']</t>
+          <t>['Qingtao Sun', 'Mingzhe Liu', 'Wuqiang Guan', 'Xiong Xiao', 'Chunyang Dong', 'Michael R. Bruchas', 'Larry S. Zweifel', 'Yulong Li', 'Lin Tian', 'Bo Li']</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -992,51 +1008,51 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.018</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>['Qingtao Sun', 'Mingzhe Liu', 'Wuqiang Guan', 'Xiong Xiao', 'Chunyang Dong', 'Michael R. Bruchas', 'Larry S. Zweifel', 'Yulong Li', 'Lin Tian', 'Bo Li']</t>
+          <t>['Lindsay A. Hohsfield', 'Sung Jin Kim', 'Rocio A. Barahona', 'Caden M. Henningfield', 'Kimiya Mansour', 'Kristen D. Vallejo', 'Kate I. Tsourmas', 'Nellie E. Kwang', 'Yasamine Ghorbanian', 'Julio Alejandro Ayala Angulo', 'Pan Gao', 'Collin Pachow', 'Matthew A. Inlay', 'Craig M. Walsh', 'Xiangmin Xu', 'Thomas E. Lane', 'Kim N. Green']</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>['Lindsay A. Hohsfield', 'Sung Jin Kim', 'Rocio A. Barahona', 'Caden M. Henningfield', 'Kimiya Mansour', 'Kristen D. Vallejo', 'Kate I. Tsourmas', 'Nellie E. Kwang', 'Yasamine Ghorbanian', 'Julio Alejandro Ayala Angulo', 'Pan Gao', 'Collin Pachow', 'Matthew A. Inlay', 'Craig M. Walsh', 'Xiangmin Xu', 'Thomas E. Lane', 'Kim N. Green']</t>
+          <t>['Charles Ducrot', 'Adèle Drouet', 'Béatrice Tessier', 'Chloé Desquines', 'Tiffany Cloâtre', 'Rania-Cérine Mazouzi', 'Florian Levet', 'Alexandre Favereaux', 'Mathieu Letellier', 'Olivier Thoumine']</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1046,24 +1062,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
+          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2411669122</t>
+          <t>10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>['Charles Ducrot', 'Adèle Drouet', 'Béatrice Tessier', 'Chloé Desquines', 'Tiffany Cloâtre', 'Rania-Cérine Mazouzi', 'Florian Levet', 'Alexandre Favereaux', 'Mathieu Letellier', 'Olivier Thoumine']</t>
+          <t>['Megan M. Davis', 'Mackenzie Woodburn', 'Tehila Nugiel', 'Divyangana Rakesh', 'Maresa Tate', 'William Asciutto', 'Weili Lin', 'Jessica R. Cohen', 'Margaret A. Sheridan']</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1073,24 +1089,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2418176122</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>['Megan M. Davis', 'Mackenzie Woodburn', 'Tehila Nugiel', 'Divyangana Rakesh', 'Maresa Tate', 'William Asciutto', 'Weili Lin', 'Jessica R. Cohen', 'Margaret A. Sheridan']</t>
+          <t>['Karthik Srinivasan', 'Eric Lowet', 'Bruno Gomes', 'Robert Desimone']</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1100,78 +1116,78 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>['Karthik Srinivasan', 'Eric Lowet', 'Bruno Gomes', 'Robert Desimone']</t>
+          <t>['Wei Wen', 'Adriana M. Prada', 'Gina G. Turrigiano']</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
+          <t>Grouping signals in primate visual cortex</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2504775122</t>
+          <t>10.1016/j.neuron.2025.05.003</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>['Wei Wen', 'Adriana M. Prada', 'Gina G. Turrigiano']</t>
+          <t>['Tom P. Franken', 'John H. Reynolds']</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Grouping signals in primate visual cortex</t>
+          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.003</t>
+          <t>10.1038/s41398-025-03398-0</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>['Tom P. Franken', 'John H. Reynolds']</t>
+          <t>['Francesca McEwan', 'Chiho Kambara', 'Jarred M. Lorusso', 'Michael K. Harte', 'Jocelyn D. Glazier', 'Reinmar Hager']</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1181,24 +1197,24 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03398-0</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>['Francesca McEwan', 'Chiho Kambara', 'Jarred M. Lorusso', 'Michael K. Harte', 'Jocelyn D. Glazier', 'Reinmar Hager']</t>
+          <t>['Omar Soler-Cedeno', 'Ewa Galaj', 'Benjamin Klein', 'Jianjing Cao', 'Guo-Hua Bi', 'Amy Hauck Newman', 'Zheng-Xiong Xi']</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1208,24 +1224,24 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1038/s41398-025-03401-8</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>['Omar Soler-Cedeno', 'Ewa Galaj', 'Benjamin Klein', 'Jianjing Cao', 'Guo-Hua Bi', 'Amy Hauck Newman', 'Zheng-Xiong Xi']</t>
+          <t>['Andreas Walther', 'Lukas Eggenberger', 'Rudolf Debelak', 'Clemens Kirschbaum', 'Isabelle Häberling', 'Ester Osuna', 'Michael Strumberger', 'Susanne Walitza', 'Jeannine Baumgartner', 'Isabelle Herter-Aeberli', 'Gregor Berger']</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1235,24 +1251,24 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
+          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03401-8</t>
+          <t>10.1038/s41398-025-03390-8</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>['Andreas Walther', 'Lukas Eggenberger', 'Rudolf Debelak', 'Clemens Kirschbaum', 'Isabelle Häberling', 'Ester Osuna', 'Michael Strumberger', 'Susanne Walitza', 'Jeannine Baumgartner', 'Isabelle Herter-Aeberli', 'Gregor Berger']</t>
+          <t>['Claire A. Lavalley', 'Marishka M. Mehta', 'Samuel Taylor', 'Anne E. Chuning', 'Jennifer L. Stewart', 'Quentin J. M. Huys', 'Sahib S. Khalsa', 'Martin P. Paulus', 'Ryan Smith']</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1262,17 +1278,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
+          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03390-8</t>
+          <t>10.1038/s41398-025-03393-5</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>['Claire A. Lavalley', 'Marishka M. Mehta', 'Samuel Taylor', 'Anne E. Chuning', 'Jennifer L. Stewart', 'Quentin J. M. Huys', 'Sahib S. Khalsa', 'Martin P. Paulus', 'Ryan Smith']</t>
+          <t>['Yi-An Hung', 'Tien-Chueh Kuo', 'Yufeng Jane Tseng', 'Chi-Yung Shang', 'Susan Shur-Fen Gau']</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1322,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1316,24 +1332,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
+          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03393-5</t>
+          <t>10.1038/s41398-025-03322-6</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>['Yi-An Hung', 'Tien-Chueh Kuo', 'Yufeng Jane Tseng', 'Chi-Yung Shang', 'Susan Shur-Fen Gau']</t>
+          <t>['Yanzhi Li', 'Liwan Zhu', 'Yang Yang', 'Caiyun Zhang', 'Hao Zhao', 'Jingman Shi', 'Wenjian Lai', 'Wenjing Zhou', 'Guangduoji Shi', 'Wanxin Wang', 'Lan Guo', 'Ciyong Lu']</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1343,24 +1359,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
+          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03322-6</t>
+          <t>10.1038/s41398-025-03399-z</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>['Yanzhi Li', 'Liwan Zhu', 'Yang Yang', 'Caiyun Zhang', 'Hao Zhao', 'Jingman Shi', 'Wenjian Lai', 'Wenjing Zhou', 'Guangduoji Shi', 'Wanxin Wang', 'Lan Guo', 'Ciyong Lu']</t>
+          <t>['Veronica Rivi', 'Pierfrancesco Sarti', 'Istvan Fodor', 'Zsolt Pirger', 'Joris M. Koene', 'Luca Pani', 'Anuradha Batabyal', 'Ken Lukowiak', 'Johanna Maria Catharina Blom', 'Fabio Tascedda', 'Cristina Benatti']</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1370,24 +1386,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
+          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03399-z</t>
+          <t>10.1038/s41398-025-03392-6</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>['Veronica Rivi', 'Pierfrancesco Sarti', 'Istvan Fodor', 'Zsolt Pirger', 'Joris M. Koene', 'Luca Pani', 'Anuradha Batabyal', 'Ken Lukowiak', 'Johanna Maria Catharina Blom', 'Fabio Tascedda', 'Cristina Benatti']</t>
+          <t>['Christelle Langley', 'Graham K. Murray', 'Sophia Armand', 'Franziska Knolle', 'Rudolf N. Cardinal', 'Annette Johansen', 'Peter S. Jensen', 'Jianfeng Feng', 'Dea S. Stenbæk', 'Gitte M. Knudsen', 'Patrick M. Fisher', 'Barbara J. Sahakian']</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1397,62 +1413,78 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
+          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03392-6</t>
+          <t>10.1038/s41398-025-03272-z</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>['Christelle Langley', 'Graham K. Murray', 'Sophia Armand', 'Franziska Knolle', 'Rudolf N. Cardinal', 'Annette Johansen', 'Peter S. Jensen', 'Jianfeng Feng', 'Dea S. Stenbæk', 'Gitte M. Knudsen', 'Patrick M. Fisher', 'Barbara J. Sahakian']</t>
+          <t>['Maryse J. Luijendijk', 'Margot E. T. Tesselaar', 'Huub H. van Rossum', 'Martijn van Faassen', 'Catharina M. Korse', 'Wieke H. M. Verbeek', 'Jocelyn R. Spruit', 'Pernilla C. Scheelings', 'Eva H. Hooghiemstra', 'Ido P. Kema', 'Henricus G. Ruhé', 'Sanne B. Schagen', 'Froukje E. de Vries']</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03272-z</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>['Maryse J. Luijendijk', 'Margot E. T. Tesselaar', 'Huub H. van Rossum', 'Martijn van Faassen', 'Catharina M. Korse', 'Wieke H. M. Verbeek', 'Jocelyn R. Spruit', 'Pernilla C. Scheelings', 'Eva H. Hooghiemstra', 'Ido P. Kema', 'Henricus G. Ruhé', 'Sanne B. Schagen', 'Froukje E. de Vries']</t>
+          <t>['Isaac Kauvar', 'Ethan B. Richman', 'Tony X. Liu', 'Chelsea Li', 'Sam Vesuna', 'Adelaida Chibukhchyan', 'Lisa Yamada', 'Adam Fogarty', 'Ethan Solomon', 'Eun Young Choi', 'Leili Mortazavi', 'Gustavo Chau Loo Kung', 'Pavithra Mukunda', 'Cephra Raja', 'Dariana Gil-Hernández', 'Kishandra Patron', 'Xue Zhang', 'Jacob Brawer', 'Shenandoah Wrobel', 'Zoe Lusk', 'Dian Lyu', 'Anish Mitra', 'Laura Hack', 'Liqun Luo', 'Logan Grosenick', 'Peter van Roessel', 'Leanne M. Williams', 'Boris D. Heifets', 'Jaimie M. Henderson', 'Jennifer A. McNab', 'Carolyn I. Rodríguez', 'Vivek Buch', 'Paul Nuyujukian', 'Karl Deisseroth']</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>10.1038/s41586-025-08746-0</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>['Aljoscha Nern', 'Frank Loesche', 'Shin-ya Takemura', 'Laura E. Burnett', 'Marisa Dreher', 'Eyal Gruntman', 'Judith Hoeller', 'Gary B. Huang', 'Michał Januszewski', 'Nathan C. Klapoetke', 'Sanna Koskela', 'Kit D. Longden', 'Zhiyuan Lu', 'Stephan Preibisch', 'Wei Qiu', 'Edward M. Rogers', 'Pavithraa Seenivasan', 'Arthur Zhao', 'John Bogovic', 'Brandon S. Canino', 'Jody Clements', 'Michael Cook', 'Samantha Finley-May', 'Miriam A. Flynn', 'Imran Hameed', 'Alexandra M. C. Fragniere', 'Kenneth J. Hayworth', 'Gary Patrick Hopkins', 'Philip M. Hubbard', 'William T. Katz', 'Julie Kovalyak', 'Shirley A. Lauchie', 'Meghan Leonard', 'Alanna Lohff', 'Charli A. Maldonado', 'Caroline Mooney', 'Nneoma Okeoma', 'Donald J. Olbris', 'Christopher Ordish', 'Tyler Paterson', 'Emily M. Phillips', 'Tobias Pietzsch', 'Jennifer Rivas Salinas', 'Patricia K. Rivlin', 'Philipp Schlegel', 'Ashley L. Scott', 'Louis A. Scuderi', 'Satoko Takemura', 'Iris Talebi', 'Alexander Thomson', 'Eric T. Trautman', 'Lowell Umayam', 'Claire Walsh', 'John J. Walsh', 'C. Shan Xu', 'Emily A. Yakal', 'Tansy Yang', 'Ting Zhao', 'Jan Funke', 'Reed George', 'Harald F. Hess', 'Gregory S. X. E. Jefferis', 'Christopher Knecht', 'Wyatt Korff', 'Stephen M. Plaza', 'Sandro Romani', 'Stephan Saalfeld', 'Louis K. Scheffer', 'Stuart Berg', 'Gerald M. Rubin', 'Michael B. Reiser']</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1462,51 +1494,51 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Psychedelic control of neuroimmune interactions governing fear</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1038/s41586-025-08880-9</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>['Aljoscha Nern', 'Frank Loesche', 'Shin-ya Takemura', 'Laura E. Burnett', 'Marisa Dreher', 'Eyal Gruntman', 'Judith Hoeller', 'Gary B. Huang', 'Michał Januszewski', 'Nathan C. Klapoetke', 'Sanna Koskela', 'Kit D. Longden', 'Zhiyuan Lu', 'Stephan Preibisch', 'Wei Qiu', 'Edward M. Rogers', 'Pavithraa Seenivasan', 'Arthur Zhao', 'John Bogovic', 'Brandon S. Canino', 'Jody Clements', 'Michael Cook', 'Samantha Finley-May', 'Miriam A. Flynn', 'Imran Hameed', 'Alexandra M. C. Fragniere', 'Kenneth J. Hayworth', 'Gary Patrick Hopkins', 'Philip M. Hubbard', 'William T. Katz', 'Julie Kovalyak', 'Shirley A. Lauchie', 'Meghan Leonard', 'Alanna Lohff', 'Charli A. Maldonado', 'Caroline Mooney', 'Nneoma Okeoma', 'Donald J. Olbris', 'Christopher Ordish', 'Tyler Paterson', 'Emily M. Phillips', 'Tobias Pietzsch', 'Jennifer Rivas Salinas', 'Patricia K. Rivlin', 'Philipp Schlegel', 'Ashley L. Scott', 'Louis A. Scuderi', 'Satoko Takemura', 'Iris Talebi', 'Alexander Thomson', 'Eric T. Trautman', 'Lowell Umayam', 'Claire Walsh', 'John J. Walsh', 'C. Shan Xu', 'Emily A. Yakal', 'Tansy Yang', 'Ting Zhao', 'Jan Funke', 'Reed George', 'Harald F. Hess', 'Gregory S. X. E. Jefferis', 'Christopher Knecht', 'Wyatt Korff', 'Stephen M. Plaza', 'Sandro Romani', 'Stephan Saalfeld', 'Louis K. Scheffer', 'Stuart Berg', 'Gerald M. Rubin', 'Michael B. Reiser']</t>
+          <t>['Elizabeth N. Chung', 'Jinsu Lee', 'Carolina M. Polonio', 'Joshua Choi', 'Camilo Faust Akl', 'Michael Kilian', 'Wiebke M. Weiß', 'Georgia Gunner', 'Mingyu Ye', 'Tae Hyun Heo', 'Sienna S. Drake', 'Liu Yang', 'Catarina R. G. L. d’Eca', 'Joon-Hyuk Lee', 'Liwen Deng', 'Daniel Farrenkopf', 'Anton M. Schüle', 'Hong-Gyun Lee', 'Oreoluwa Afolabi', 'Sharmin Ghaznavi', 'Stelios M. Smirnakis', 'Isaac M. Chiu', 'Vijay K. Kuchroo', 'Francisco J. Quintana', 'Michael A. Wheeler']</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Psychedelic control of neuroimmune interactions governing fear</t>
+          <t>A neural basis for distinguishing imagination from reality</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08880-9</t>
+          <t>10.1016/j.neuron.2025.05.015</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>['Elizabeth N. Chung', 'Jinsu Lee', 'Carolina M. Polonio', 'Joshua Choi', 'Camilo Faust Akl', 'Michael Kilian', 'Wiebke M. Weiß', 'Georgia Gunner', 'Mingyu Ye', 'Tae Hyun Heo', 'Sienna S. Drake', 'Liu Yang', 'Catarina R. G. L. d’Eca', 'Joon-Hyuk Lee', 'Liwen Deng', 'Daniel Farrenkopf', 'Anton M. Schüle', 'Hong-Gyun Lee', 'Oreoluwa Afolabi', 'Sharmin Ghaznavi', 'Stelios M. Smirnakis', 'Isaac M. Chiu', 'Vijay K. Kuchroo', 'Francisco J. Quintana', 'Michael A. Wheeler']</t>
+          <t>['Nadine Dijkstra', 'Thomas von Rein', 'Peter Kok', 'Stephen M. Fleming']</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1516,62 +1548,78 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>A neural basis for distinguishing imagination from reality</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.015</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>['Nadine Dijkstra', 'Thomas von Rein', 'Peter Kok', 'Stephen M. Fleming']</t>
+          <t>['Wang Zheng', 'Augustus J. Lowry', 'Harper E. Smith', 'Jiale Xie', 'Shaun Rawson', 'Chen Wang', 'Jin Ou', 'Marcos Sotomayor', 'Tian-Min Fu', 'Huanghe Yang', 'Jeffrey R. Holt']</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>['Wang Zheng', 'Augustus J. Lowry', 'Harper E. Smith', 'Jiale Xie', 'Shaun Rawson', 'Chen Wang', 'Jin Ou', 'Marcos Sotomayor', 'Tian-Min Fu', 'Huanghe Yang', 'Jeffrey R. Holt']</t>
+          <t>['Yu Zheng', 'Ruyi Cai', 'Kui Wang', 'Junwei Zhang', 'Yizhou Zhuo', 'Hui Dong', 'Yuqi Zhang', 'Yifan Wang', 'Fei Deng', 'En Ji', 'Yiwen Cui', 'Shilin Fang', 'Xinxin Zhang', 'Haiyun Huang', 'Kecheng Zhang', 'Jinxu Wang', 'Guochuan Li', 'Xiaolei Miao', 'Zhenghua Wang', 'Yuqing Yang', 'Shaochuang Li', 'Jonathan B. Grimm', 'Kai Johnsson', 'Eric R. Schreiter', 'Luke D. Lavis', 'Zhixing Chen', 'Yu Mu', 'Yulong Li']</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>The Journal of Neuroscience</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>10.1523/JNEUROSCI.1920-24.2025</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>['Rikard Frederiksen', 'Paul J. Bonezzi', 'Gordon L. Fain', 'Alapakkam P. Sampath']</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1581,24 +1629,24 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
+          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-24.2025</t>
+          <t>10.1523/JNEUROSCI.1139-24.2025</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>['Rikard Frederiksen', 'Paul J. Bonezzi', 'Gordon L. Fain', 'Alapakkam P. Sampath']</t>
+          <t>['Paula T. Kuokkanen', 'Ira Kraemer', 'Christine Köppl', 'Catherine E. Carr', 'Richard Kempter']</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1608,24 +1656,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
+          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1139-24.2025</t>
+          <t>10.1523/JNEUROSCI.0217-25.2025</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>['Paula T. Kuokkanen', 'Ira Kraemer', 'Christine Köppl', 'Catherine E. Carr', 'Richard Kempter']</t>
+          <t>['Paola Alemán-Andrade', 'Menno P. Witter', 'Ken-Ichiro Tsutsui', 'Shinya Ohara']</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1635,24 +1683,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
+          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0217-25.2025</t>
+          <t>10.1523/JNEUROSCI.2325-24.2025</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>['Paola Alemán-Andrade', 'Menno P. Witter', 'Ken-Ichiro Tsutsui', 'Shinya Ohara']</t>
+          <t>['James B. Whitley', 'Sean P. Masterson', 'Thomas Gordon', 'Kyle L. Whyland', 'Peter W. Campbell', 'Na Zhou', 'Gubbi Govindaiah', 'William Guido', 'Martha E. Bickford']</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1662,24 +1710,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
+          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2325-24.2025</t>
+          <t>10.1523/JNEUROSCI.1001-24.2025</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>['James B. Whitley', 'Sean P. Masterson', 'Thomas Gordon', 'Kyle L. Whyland', 'Peter W. Campbell', 'Na Zhou', 'Gubbi Govindaiah', 'William Guido', 'Martha E. Bickford']</t>
+          <t>['Carolina Fernandes-Henriques', 'Yuval Guetta', 'Mia G. Sclar', 'Rebecca Zhang', 'Yuka Miura', 'Katherine R. Surrence', 'Allyson K. Friedman', 'Ekaterina Likhtik']</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1689,24 +1737,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
+          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1001-24.2025</t>
+          <t>10.1523/JNEUROSCI.1876-24.2025</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>['Carolina Fernandes-Henriques', 'Yuval Guetta', 'Mia G. Sclar', 'Rebecca Zhang', 'Yuka Miura', 'Katherine R. Surrence', 'Allyson K. Friedman', 'Ekaterina Likhtik']</t>
+          <t>['Lidon Marin-Marin', 'Susanne Eisenhauer', 'Tirso R. J. Gonzalez Alam', 'Daniel S. Margulies', 'Jonathan Smallwood', 'Elizabeth Jefferies']</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1716,24 +1764,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
+          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1876-24.2025</t>
+          <t>10.1523/JNEUROSCI.2187-24.2025</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>['Lidon Marin-Marin', 'Susanne Eisenhauer', 'Tirso R. J. Gonzalez Alam', 'Daniel S. Margulies', 'Jonathan Smallwood', 'Elizabeth Jefferies']</t>
+          <t>['Min Wu', 'Marleen J. Schoenfeld', 'Carl Lindersson', 'Sven Braeutigam', 'Catharina Zich', 'Charlotte J. Stagg']</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1743,24 +1791,24 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2187-24.2025</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>['Min Wu', 'Marleen J. Schoenfeld', 'Carl Lindersson', 'Sven Braeutigam', 'Catharina Zich', 'Charlotte J. Stagg']</t>
+          <t>['Marie-Lucie Read', 'Carl J. Hodgetts', 'Andrew D. Lawrence', 'C. John Evans', 'Krish D. Singh', 'Katja Umla-Runge', 'Kim S. Graham']</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1770,24 +1818,24 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1523/JNEUROSCI.2378-24.2025</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>['Marie-Lucie Read', 'Carl J. Hodgetts', 'Andrew D. Lawrence', 'C. John Evans', 'Krish D. Singh', 'Katja Umla-Runge', 'Kim S. Graham']</t>
+          <t>['Marie Levorsen', 'Ryuta Aoki', 'Constantine Sedikides', 'Keise Izuma']</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1797,24 +1845,24 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
+          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2378-24.2025</t>
+          <t>10.1523/JNEUROSCI.0044-25.2025</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>['Marie Levorsen', 'Ryuta Aoki', 'Constantine Sedikides', 'Keise Izuma']</t>
+          <t>['Puti Wen', 'Lowell W. Thompson', 'Ari Rosenberg', 'Michael S. Landy', 'Bas Rokers']</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1824,24 +1872,24 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
+          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0044-25.2025</t>
+          <t>10.1523/JNEUROSCI.2186-24.2025</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>['Puti Wen', 'Lowell W. Thompson', 'Ari Rosenberg', 'Michael S. Landy', 'Bas Rokers']</t>
+          <t>['Siyi Chen (陈思佚)', 'Nika Merkuš', 'Shao-Yang Tsai (蔡劭扬)', 'Si Cheng (程思)', 'Hermann J. Müller', 'Zhuanghua Shi (施壮华)']</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1851,24 +1899,24 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2186-24.2025</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>['Siyi Chen (陈思佚)', 'Nika Merkuš', 'Shao-Yang Tsai (蔡劭扬)', 'Si Cheng (程思)', 'Hermann J. Müller', 'Zhuanghua Shi (施壮华)']</t>
+          <t>['Reut Hazani', 'Jocelyn M. Breton', 'Estherina Trachtenberg', 'Keren Ruzal', 'Bar Shvalbo', 'Ben Kantor', 'Adva Maman', 'Einat Bigelman', 'Steve Cole', 'Aron Weller', 'Inbal Ben-Ami Bartal']</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1878,24 +1926,24 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>['Reut Hazani', 'Jocelyn M. Breton', 'Estherina Trachtenberg', 'Keren Ruzal', 'Bar Shvalbo', 'Ben Kantor', 'Adva Maman', 'Einat Bigelman', 'Steve Cole', 'Aron Weller', 'Inbal Ben-Ami Bartal']</t>
+          <t>['Yan Chen', 'Xiangyue Xiao', 'Zhicai Dong', 'Junhua Ding', 'Sara Cruz', 'Ming Zhang', 'Yuhan Lu', 'Nai Ding', 'Charlène Aubinet', 'Steven Laureys', 'Haibo Di']</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1905,51 +1953,51 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>['Yan Chen', 'Xiangyue Xiao', 'Zhicai Dong', 'Junhua Ding', 'Sara Cruz', 'Ming Zhang', 'Yuhan Lu', 'Nai Ding', 'Charlène Aubinet', 'Steven Laureys', 'Haibo Di']</t>
+          <t>['Sai Yasukochi', 'Wakaba Yamakawa', 'Marie Taniguchi', 'Sayaka Itoyama', 'Akito Tsuruta', 'Naoki Kusunose', 'Tomoaki Yamauchi', 'Risako Nakamura', 'Naoya Matsunaga', 'Shigehiro Ohdo', 'Satoru Koyanagi']</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>['Sai Yasukochi', 'Wakaba Yamakawa', 'Marie Taniguchi', 'Sayaka Itoyama', 'Akito Tsuruta', 'Naoki Kusunose', 'Tomoaki Yamauchi', 'Risako Nakamura', 'Naoya Matsunaga', 'Shigehiro Ohdo', 'Satoru Koyanagi']</t>
+          <t>['Xiaodong Xu', 'Cheng Jia', 'Kang Chen', 'Lijuan Chen']</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1959,42 +2007,15 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
-        <is>
-          <t>['Xiaodong Xu', 'Cheng Jia', 'Kang Chen', 'Lijuan Chen']</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>npj Science of Learning</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>10.1038/s41539-025-00308-3</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
         <is>
           <t>['Christoph Bamberg', 'Sarah Weigelt', 'Klara Hagelweide']</t>
         </is>

</xml_diff>